<commit_message>
feat(batch): include Variable 7 (Tenure) in Paper 234 effect sizes (ES ID 6, r=0.14)
</commit_message>
<xml_diff>
--- a/03_Coding_Sheets/234_235_236_238.xlsx
+++ b/03_Coding_Sheets/234_235_236_238.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AX11"/>
+  <dimension ref="A1:AX12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1425,16 +1425,140 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>235</v>
+        <v>234</v>
+      </c>
+      <c r="D9" t="n">
+        <v>6</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>0 = exclude</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level (team/firm/org analysis)</t>
+          <t>1 = include</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>1 = Cross-sectional design</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>Taiwan</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>0 = Domestic</t>
+        </is>
+      </c>
+      <c r="V9" t="n">
+        <v>124</v>
+      </c>
+      <c r="W9" t="n">
+        <v>999</v>
+      </c>
+      <c r="X9" t="n">
+        <v>999</v>
+      </c>
+      <c r="Y9" t="n">
+        <v>999</v>
+      </c>
+      <c r="Z9" t="inlineStr">
+        <is>
+          <t>Software company employees and supervisors across 12 functional units</t>
+        </is>
+      </c>
+      <c r="AA9" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB9" t="n">
+        <v>999</v>
+      </c>
+      <c r="AC9" t="n">
+        <v>999</v>
+      </c>
+      <c r="AD9" t="inlineStr">
+        <is>
+          <t>3 = Others</t>
+        </is>
+      </c>
+      <c r="AE9" t="inlineStr">
+        <is>
+          <t>Sociometric peer nominations: respondents nominated up to five contacts for work-related advice to calculate in-degree centrality for intra- and inter-department contacts; boundary spanners were defined as individuals in the top third of both intra-department and external communication distributions following Tushman &amp; Scanlan (1981b).</t>
+        </is>
+      </c>
+      <c r="AF9" t="inlineStr">
+        <is>
+          <t>Sparrowe (2001)</t>
+        </is>
+      </c>
+      <c r="AG9" t="inlineStr">
+        <is>
+          <t>Operationalized as a two-step boundary spanner following Tushman &amp; Scanlan (1981b): individuals who are both internal communication stars (top third of intra-department advice communication distribution) and external communication stars (top third of inter-department advice communication distribution) based on sociometric advice nominations.</t>
+        </is>
+      </c>
+      <c r="AH9" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI9" t="n">
+        <v>999</v>
+      </c>
+      <c r="AJ9" t="n">
+        <v>999</v>
+      </c>
+      <c r="AK9" t="inlineStr">
+        <is>
+          <t>4 = Objective</t>
+        </is>
+      </c>
+      <c r="AL9" t="inlineStr">
+        <is>
+          <t>Objective length of time a person has been with the company in years.</t>
+        </is>
+      </c>
+      <c r="AM9" t="inlineStr">
+        <is>
+          <t>length of time a person has been with the company</t>
+        </is>
+      </c>
+      <c r="AN9" t="inlineStr">
+        <is>
+          <t>Tenure was included as control variables because prior work has suggested that the length of time a person has been with the company is likely to affect his or her work performance.</t>
+        </is>
+      </c>
+      <c r="AO9" t="inlineStr">
+        <is>
+          <t>Boundary spanner</t>
+        </is>
+      </c>
+      <c r="AP9" t="n">
+        <v>999</v>
+      </c>
+      <c r="AQ9" t="n">
+        <v>999</v>
+      </c>
+      <c r="AR9" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS9" t="inlineStr">
+        <is>
+          <t>Tenure</t>
+        </is>
+      </c>
+      <c r="AT9" t="n">
+        <v>999</v>
+      </c>
+      <c r="AU9" t="n">
+        <v>999</v>
+      </c>
+      <c r="AV9" t="n">
+        <v>999</v>
+      </c>
+      <c r="AW9" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="AX9" t="inlineStr">
+        <is>
+          <t>Table 2 (p. 1141), Row: 7. Tenure, Col: 4, Raw: 0.14 | Latent correlation: [p. 1140] "To assess discriminant validity, Fornell &amp; Larcker (1981) suggested the use of Average Variance Extracted (AVE), which should be greater than the variances shared between the construct. The comparison can be made in the correlation matrix (see Table 2), including the correlations between different constructs in the off-diagonal elements of the matrix, and the square roots of the AVE for each of the constructs along the diagonal."</t>
         </is>
       </c>
     </row>
@@ -1445,7 +1569,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -1465,14 +1589,34 @@
         </is>
       </c>
       <c r="B11" t="n">
+        <v>236</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>0 = exclude</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
         <v>238</v>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>0 = exclude</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>1 = No effect size of interest</t>
         </is>

</xml_diff>

<commit_message>
chore: optimize BSMA repository, master architectural map, coding sheets, and script suite (V5.4)
</commit_message>
<xml_diff>
--- a/03_Coding_Sheets/234_235_236_238.xlsx
+++ b/03_Coding_Sheets/234_235_236_238.xlsx
@@ -783,7 +783,7 @@
       </c>
       <c r="AG4" t="inlineStr">
         <is>
-          <t>Operationalized as a two-step boundary spanner following Tushman &amp; Scanlan (1981b): individuals who are both internal communication stars (top third of intra-department advice communication distribution) and external communication stars (top third of inter-department advice communication distribution) based on sociometric advice nominations.</t>
+          <t>[Methodology, p. 1138] "To assess the network relations, we follow the work of Sparrowe (2001) by asking the respondents one question: 'Who do you go to for help or advice on work-related matters?'" Operationalized as a two-step boundary spanner following Tushman &amp; Scanlan (1981b): individuals who are both internal communication stars (top third of intra-department advice communication distribution) and external communication stars (top third of inter-department advice communication distribution) based on sociometric advice nominations.</t>
         </is>
       </c>
       <c r="AH4" t="n">
@@ -812,7 +812,7 @@
       </c>
       <c r="AN4" t="inlineStr">
         <is>
-          <t>Single-item sociometric measure assessing intellectual capability by calculating in-degree centrality of peer nominations of the most competent persons in the company.</t>
+          <t>[Methodology, p. 1139] "Following the work of Tushman &amp; Scanlan (1981a), we used one question to assess the level of intellectual capability of individuals." Single-item sociometric measure assessing intellectual capability by calculating in-degree centrality of peer nominations of the most competent persons in the company.</t>
         </is>
       </c>
       <c r="AO4" t="inlineStr">
@@ -927,7 +927,7 @@
       </c>
       <c r="AG5" t="inlineStr">
         <is>
-          <t>Operationalized as a two-step boundary spanner following Tushman &amp; Scanlan (1981b): individuals who are both internal communication stars (top third of intra-department advice communication distribution) and external communication stars (top third of inter-department advice communication distribution) based on sociometric advice nominations.</t>
+          <t>[Methodology, p. 1138] "To assess the network relations, we follow the work of Sparrowe (2001) by asking the respondents one question: 'Who do you go to for help or advice on work-related matters?'" Operationalized as a two-step boundary spanner following Tushman &amp; Scanlan (1981b): individuals who are both internal communication stars (top third of intra-department advice communication distribution) and external communication stars (top third of inter-department advice communication distribution) based on sociometric advice nominations.</t>
         </is>
       </c>
       <c r="AH5" t="n">
@@ -956,7 +956,7 @@
       </c>
       <c r="AN5" t="inlineStr">
         <is>
-          <t>Two-item sociometric measure developed by the authors to assess interpersonal trusting relationships by calculating in-degree centrality of peer nominations.</t>
+          <t>[Methodology, p. 1139] "We developed two questions to examine the inter-personal trusting relationships in the company: (1) 'Please indicate whom you can rely on without any fear that they will take advantage of you' and (2) 'In general, who will always keep the promises they make to you?'" Two-item sociometric measure developed by the authors to assess interpersonal trusting relationships by calculating in-degree centrality of peer nominations.</t>
         </is>
       </c>
       <c r="AO5" t="inlineStr">
@@ -1071,7 +1071,7 @@
       </c>
       <c r="AG6" t="inlineStr">
         <is>
-          <t>Operationalized as a two-step boundary spanner following Tushman &amp; Scanlan (1981b): individuals who are both internal communication stars (top third of intra-department advice communication distribution) and external communication stars (top third of inter-department advice communication distribution) based on sociometric advice nominations.</t>
+          <t>[Methodology, p. 1138] "To assess the network relations, we follow the work of Sparrowe (2001) by asking the respondents one question: 'Who do you go to for help or advice on work-related matters?'" Operationalized as a two-step boundary spanner following Tushman &amp; Scanlan (1981b): individuals who are both internal communication stars (top third of intra-department advice communication distribution) and external communication stars (top third of inter-department advice communication distribution) based on sociometric advice nominations.</t>
         </is>
       </c>
       <c r="AH6" t="n">
@@ -1215,7 +1215,7 @@
       </c>
       <c r="AG7" t="inlineStr">
         <is>
-          <t>Operationalized as a two-step boundary spanner following Tushman &amp; Scanlan (1981b): individuals who are both internal communication stars (top third of intra-department advice communication distribution) and external communication stars (top third of inter-department advice communication distribution) based on sociometric advice nominations.</t>
+          <t>[Methodology, p. 1138] "To assess the network relations, we follow the work of Sparrowe (2001) by asking the respondents one question: 'Who do you go to for help or advice on work-related matters?'" Operationalized as a two-step boundary spanner following Tushman &amp; Scanlan (1981b): individuals who are both internal communication stars (top third of intra-department advice communication distribution) and external communication stars (top third of inter-department advice communication distribution) based on sociometric advice nominations.</t>
         </is>
       </c>
       <c r="AH7" t="n">
@@ -1239,7 +1239,7 @@
       </c>
       <c r="AN7" t="inlineStr">
         <is>
-          <t>Three-item scale rated by direct supervisors on a 5-point Likert format adapted from Mehra et al. (2001).</t>
+          <t>[Methodology, p. 1139] "Following prior research (Mehra et al., 2001), supervisors related subordinates' innovativeness on three items." Three-item scale rated by direct supervisors on a 5-point Likert format adapted from Mehra et al. (2001).</t>
         </is>
       </c>
       <c r="AO7" t="inlineStr">
@@ -1354,7 +1354,7 @@
       </c>
       <c r="AG8" t="inlineStr">
         <is>
-          <t>Operationalized as a two-step boundary spanner following Tushman &amp; Scanlan (1981b): individuals who are both internal communication stars (top third of intra-department advice communication distribution) and external communication stars (top third of inter-department advice communication distribution) based on sociometric advice nominations.</t>
+          <t>[Methodology, p. 1138] "To assess the network relations, we follow the work of Sparrowe (2001) by asking the respondents one question: 'Who do you go to for help or advice on work-related matters?'" Operationalized as a two-step boundary spanner following Tushman &amp; Scanlan (1981b): individuals who are both internal communication stars (top third of intra-department advice communication distribution) and external communication stars (top third of inter-department advice communication distribution) based on sociometric advice nominations.</t>
         </is>
       </c>
       <c r="AH8" t="n">
@@ -1378,7 +1378,7 @@
       </c>
       <c r="AN8" t="inlineStr">
         <is>
-          <t>Three-item scale rated by direct supervisors on a 5-point Likert format adapted from Mehra et al. (2001) measuring overall job performance, likelihood of future career success, and succession likelihood.</t>
+          <t>[Methodology, p. 1139] "Following prior research (Mehra et al., 2001), supervisors related subordinates' innovativeness on three items." Three-item scale rated by direct supervisors on a 5-point Likert format adapted from Mehra et al. (2001) measuring overall job performance, likelihood of future career success, and succession likelihood.</t>
         </is>
       </c>
       <c r="AO8" t="inlineStr">
@@ -1493,7 +1493,7 @@
       </c>
       <c r="AG9" t="inlineStr">
         <is>
-          <t>Operationalized as a two-step boundary spanner following Tushman &amp; Scanlan (1981b): individuals who are both internal communication stars (top third of intra-department advice communication distribution) and external communication stars (top third of inter-department advice communication distribution) based on sociometric advice nominations.</t>
+          <t>[Methodology, p. 1138] "To assess the network relations, we follow the work of Sparrowe (2001) by asking the respondents one question: 'Who do you go to for help or advice on work-related matters?'" Operationalized as a two-step boundary spanner following Tushman &amp; Scanlan (1981b): individuals who are both internal communication stars (top third of intra-department advice communication distribution) and external communication stars (top third of inter-department advice communication distribution) based on sociometric advice nominations.</t>
         </is>
       </c>
       <c r="AH9" t="n">

</xml_diff>